<commit_message>
v4 rodado- com 1300+ metafeatures
</commit_message>
<xml_diff>
--- a/intermidiate_tables_csv/04_outer_cv_results.xlsx
+++ b/intermidiate_tables_csv/04_outer_cv_results.xlsx
@@ -480,28 +480,28 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>79</v>
+        <v>955</v>
       </c>
       <c r="C2" t="n">
-        <v>23</v>
+        <v>461</v>
       </c>
       <c r="D2" t="n">
-        <v>70.88607594936708</v>
+        <v>51.72774869109949</v>
       </c>
       <c r="E2" t="n">
-        <v>0.661089273292953</v>
+        <v>0.642011400207719</v>
       </c>
       <c r="F2" t="n">
-        <v>0.6031746031746031</v>
+        <v>0.6507936507936508</v>
       </c>
       <c r="G2" t="n">
-        <v>0.5873015873015873</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="H2" t="n">
-        <v>0.6031746031746031</v>
+        <v>0.6507936507936508</v>
       </c>
       <c r="I2" t="n">
-        <v>0.5873015873015873</v>
+        <v>0.6190476190476191</v>
       </c>
     </row>
     <row r="3">
@@ -509,28 +509,28 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>81</v>
+        <v>954</v>
       </c>
       <c r="C3" t="n">
-        <v>27</v>
+        <v>462</v>
       </c>
       <c r="D3" t="n">
-        <v>66.66666666666667</v>
+        <v>51.57232704402516</v>
       </c>
       <c r="E3" t="n">
-        <v>0.6390867579908676</v>
+        <v>0.6372462061674767</v>
       </c>
       <c r="F3" t="n">
-        <v>0.6349206349206349</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="G3" t="n">
-        <v>0.6349206349206349</v>
+        <v>0.6825396825396826</v>
       </c>
       <c r="H3" t="n">
-        <v>0.6190476190476191</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="I3" t="n">
-        <v>0.6031746031746031</v>
+        <v>0.6507936507936508</v>
       </c>
     </row>
     <row r="4">
@@ -538,19 +538,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>80</v>
+        <v>950</v>
       </c>
       <c r="C4" t="n">
-        <v>33</v>
+        <v>480</v>
       </c>
       <c r="D4" t="n">
-        <v>58.75</v>
+        <v>49.47368421052632</v>
       </c>
       <c r="E4" t="n">
-        <v>0.6338543890725871</v>
+        <v>0.6412861926339604</v>
       </c>
       <c r="F4" t="n">
-        <v>0.6507936507936508</v>
+        <v>0.6349206349206349</v>
       </c>
       <c r="G4" t="n">
         <v>0.6349206349206349</v>
@@ -567,28 +567,28 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>81</v>
+        <v>950</v>
       </c>
       <c r="C5" t="n">
-        <v>27</v>
+        <v>494</v>
       </c>
       <c r="D5" t="n">
-        <v>66.66666666666667</v>
+        <v>48</v>
       </c>
       <c r="E5" t="n">
-        <v>0.6392127224059204</v>
+        <v>0.643038150842387</v>
       </c>
       <c r="F5" t="n">
-        <v>0.6349206349206349</v>
+        <v>0.6825396825396826</v>
       </c>
       <c r="G5" t="n">
         <v>0.6984126984126984</v>
       </c>
       <c r="H5" t="n">
-        <v>0.6349206349206349</v>
+        <v>0.7301587301587301</v>
       </c>
       <c r="I5" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.7142857142857143</v>
       </c>
     </row>
     <row r="6">
@@ -596,28 +596,28 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>82</v>
+        <v>947</v>
       </c>
       <c r="C6" t="n">
-        <v>22</v>
+        <v>468</v>
       </c>
       <c r="D6" t="n">
-        <v>73.17073170731707</v>
+        <v>50.58078141499471</v>
       </c>
       <c r="E6" t="n">
-        <v>0.6474863570553513</v>
+        <v>0.6241146997153088</v>
       </c>
       <c r="F6" t="n">
+        <v>0.5967741935483871</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.6129032258064516</v>
+      </c>
+      <c r="H6" t="n">
         <v>0.5645161290322581</v>
       </c>
-      <c r="G6" t="n">
-        <v>0.5806451612903226</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0.6451612903225806</v>
-      </c>
       <c r="I6" t="n">
-        <v>0.5806451612903226</v>
+        <v>0.5483870967741935</v>
       </c>
     </row>
     <row r="7">
@@ -625,25 +625,25 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>81</v>
+        <v>953</v>
       </c>
       <c r="C7" t="n">
-        <v>25</v>
+        <v>458</v>
       </c>
       <c r="D7" t="n">
-        <v>69.1358024691358</v>
+        <v>51.94123819517313</v>
       </c>
       <c r="E7" t="n">
-        <v>0.6442584136648063</v>
+        <v>0.6381937784430978</v>
       </c>
       <c r="F7" t="n">
         <v>0.6451612903225806</v>
       </c>
       <c r="G7" t="n">
-        <v>0.5806451612903226</v>
+        <v>0.6451612903225806</v>
       </c>
       <c r="H7" t="n">
-        <v>0.6290322580645161</v>
+        <v>0.6129032258064516</v>
       </c>
       <c r="I7" t="n">
         <v>0.6290322580645161</v>
@@ -654,28 +654,28 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>81</v>
+        <v>950</v>
       </c>
       <c r="C8" t="n">
-        <v>34</v>
+        <v>329</v>
       </c>
       <c r="D8" t="n">
-        <v>58.0246913580247</v>
+        <v>65.36842105263159</v>
       </c>
       <c r="E8" t="n">
-        <v>0.6414535522274628</v>
+        <v>0.6206965633261234</v>
       </c>
       <c r="F8" t="n">
-        <v>0.6774193548387096</v>
+        <v>0.6290322580645161</v>
       </c>
       <c r="G8" t="n">
         <v>0.6612903225806451</v>
       </c>
       <c r="H8" t="n">
-        <v>0.6129032258064516</v>
+        <v>0.6290322580645161</v>
       </c>
       <c r="I8" t="n">
-        <v>0.5967741935483871</v>
+        <v>0.6612903225806451</v>
       </c>
     </row>
     <row r="9">
@@ -683,25 +683,25 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>81</v>
+        <v>950</v>
       </c>
       <c r="C9" t="n">
-        <v>28</v>
+        <v>402</v>
       </c>
       <c r="D9" t="n">
-        <v>65.4320987654321</v>
+        <v>57.68421052631578</v>
       </c>
       <c r="E9" t="n">
-        <v>0.6138981904278707</v>
+        <v>0.5980511802071871</v>
       </c>
       <c r="F9" t="n">
         <v>0.7419354838709677</v>
       </c>
       <c r="G9" t="n">
-        <v>0.7419354838709677</v>
+        <v>0.7903225806451613</v>
       </c>
       <c r="H9" t="n">
-        <v>0.7096774193548387</v>
+        <v>0.8064516129032258</v>
       </c>
       <c r="I9" t="n">
         <v>0.7741935483870968</v>

</xml_diff>